<commit_message>
[auto-snapshot] 2026-04-27 04:00 | onda-hompage | 49 files
</commit_message>
<xml_diff>
--- a/naver-place-crawler/results_health/전주_PT.xlsx
+++ b/naver-place-crawler/results_health/전주_PT.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V189"/>
+  <dimension ref="A1:V202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -18136,6 +18136,1228 @@
         </is>
       </c>
     </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>헬스장</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>바디포커스 운동&amp;재활센터 LH점</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>huswl1214@naver.com</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr"/>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>0507-1305-8931</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr"/>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>전북특별자치도 전주시 완산구 호암로 84 3층 바디포커스 LH점</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/huswl1214/223893338680</t>
+        </is>
+      </c>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J190" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K190" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="L190" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M190" t="inlineStr"/>
+      <c r="N190" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O190" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P190" t="n">
+        <v>37</v>
+      </c>
+      <c r="Q190" t="n">
+        <v>63</v>
+      </c>
+      <c r="R190" t="n">
+        <v>100</v>
+      </c>
+      <c r="S190" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T190" t="inlineStr">
+        <is>
+          <t>1813815685</t>
+        </is>
+      </c>
+      <c r="U190" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1813815685</t>
+        </is>
+      </c>
+      <c r="V190" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>스포츠시설</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>모이라짐 신시가지점</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>moiragym@naver.com</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr"/>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>0507-1498-9102</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr"/>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>전북특별자치도 전주시 완산구 홍산중앙로 18 7층</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/moiragym</t>
+        </is>
+      </c>
+      <c r="I191" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J191" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K191" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="L191" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M191" t="inlineStr"/>
+      <c r="N191" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O191" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P191" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q191" t="n">
+        <v>174</v>
+      </c>
+      <c r="R191" t="n">
+        <v>186</v>
+      </c>
+      <c r="S191" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T191" t="inlineStr">
+        <is>
+          <t>36960147</t>
+        </is>
+      </c>
+      <c r="U191" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/36960147</t>
+        </is>
+      </c>
+      <c r="V191" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>스포츠센터</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>좋음PT</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>kkk43211@naver.com</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>themosttimes@tmt.co.kr</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>063-223-8231</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr"/>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>전북특별자치도 전주시 완산구 강변로 70 로드빌딩2층 좋음PT</t>
+        </is>
+      </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>https://www.themosttimes.co.kr/43119</t>
+        </is>
+      </c>
+      <c r="I192" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J192" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K192" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L192" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M192" t="inlineStr"/>
+      <c r="N192" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O192" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P192" t="n">
+        <v>151</v>
+      </c>
+      <c r="Q192" t="n">
+        <v>308</v>
+      </c>
+      <c r="R192" t="n">
+        <v>459</v>
+      </c>
+      <c r="S192" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T192" t="inlineStr">
+        <is>
+          <t>1582951760</t>
+        </is>
+      </c>
+      <c r="U192" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1582951760</t>
+        </is>
+      </c>
+      <c r="V192" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>스포츠시설</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>제로백 PT 반월 7호점</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>zeroback2022@naver.com</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr"/>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>0507-1382-0125</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr"/>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>전북특별자치도 전주시 덕진구 쪽구름로 124 4층 제로백피트니스</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/zeroback2022/223821074759</t>
+        </is>
+      </c>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J193" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K193" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="L193" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M193" t="inlineStr"/>
+      <c r="N193" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O193" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P193" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q193" t="n">
+        <v>2</v>
+      </c>
+      <c r="R193" t="n">
+        <v>7</v>
+      </c>
+      <c r="S193" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T193" t="inlineStr">
+        <is>
+          <t>2082432764</t>
+        </is>
+      </c>
+      <c r="U193" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/2082432764</t>
+        </is>
+      </c>
+      <c r="V193" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>헬스장</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>24시 헬스 PT 제로백피트니스 반월점</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>zeroback2022@naver.com</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr"/>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>0507-1438-8873</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr"/>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>전북특별자치도 전주시 덕진구 쪽구름로 124 4층 401호</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/zeroback2022/223794709810</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J194" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K194" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="L194" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M194" t="inlineStr"/>
+      <c r="N194" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O194" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P194" t="n">
+        <v>492</v>
+      </c>
+      <c r="Q194" t="n">
+        <v>73</v>
+      </c>
+      <c r="R194" t="n">
+        <v>565</v>
+      </c>
+      <c r="S194" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T194" t="inlineStr">
+        <is>
+          <t>1691197101</t>
+        </is>
+      </c>
+      <c r="U194" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1691197101</t>
+        </is>
+      </c>
+      <c r="V194" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>헬스장</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>온탑피트니스 만성점</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>ontopfit@naver.com</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr"/>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>0507-1355-5810</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr"/>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>전북특별자치도 전주시 덕진구 만성중앙로 76 4층 온탑피트니스</t>
+        </is>
+      </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/ontopfit</t>
+        </is>
+      </c>
+      <c r="I195" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J195" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K195" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="L195" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M195" t="inlineStr"/>
+      <c r="N195" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O195" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P195" t="n">
+        <v>175</v>
+      </c>
+      <c r="Q195" t="n">
+        <v>280</v>
+      </c>
+      <c r="R195" t="n">
+        <v>455</v>
+      </c>
+      <c r="S195" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T195" t="inlineStr">
+        <is>
+          <t>1089561368</t>
+        </is>
+      </c>
+      <c r="U195" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1089561368</t>
+        </is>
+      </c>
+      <c r="V195" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>무예,격투기</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>퍼스트짐 서신본관</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>z1x2a3s4@naver.com</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr"/>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>0507-1401-3222</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr"/>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>전북특별자치도 전주시 완산구 새터로 52-7 광진장미아파트 상가2층</t>
+        </is>
+      </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>http://instagram.com/firstgym_jiujitsu</t>
+        </is>
+      </c>
+      <c r="I196" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J196" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K196" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L196" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M196" t="inlineStr"/>
+      <c r="N196" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O196" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P196" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q196" t="n">
+        <v>106</v>
+      </c>
+      <c r="R196" t="n">
+        <v>116</v>
+      </c>
+      <c r="S196" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T196" t="inlineStr">
+        <is>
+          <t>1616064720</t>
+        </is>
+      </c>
+      <c r="U196" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1616064720</t>
+        </is>
+      </c>
+      <c r="V196" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>스포츠시설</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>헬스챌린저</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>rkdgml1817@naver.com</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr"/>
+      <c r="E197" t="inlineStr"/>
+      <c r="F197" t="inlineStr"/>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>전북특별자치도 전주시 덕진구 백제대로 555 B1층 헬스챌린저</t>
+        </is>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/rkdgml1817</t>
+        </is>
+      </c>
+      <c r="I197" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J197" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K197" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="L197" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M197" t="inlineStr"/>
+      <c r="N197" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O197" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P197" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q197" t="n">
+        <v>21</v>
+      </c>
+      <c r="R197" t="n">
+        <v>33</v>
+      </c>
+      <c r="S197" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T197" t="inlineStr">
+        <is>
+          <t>1642194859</t>
+        </is>
+      </c>
+      <c r="U197" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1642194859</t>
+        </is>
+      </c>
+      <c r="V197" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>헬스장</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>골드피티짐</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>superwoo1@naver.com</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr"/>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>070-7869-9976</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr"/>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>전북특별자치도 전주시 덕진구 조경단로 33-1 2층</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I198" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J198" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K198" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L198" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M198" t="inlineStr"/>
+      <c r="N198" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O198" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P198" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q198" t="n">
+        <v>291</v>
+      </c>
+      <c r="R198" t="n">
+        <v>291</v>
+      </c>
+      <c r="S198" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T198" t="inlineStr">
+        <is>
+          <t>20662679</t>
+        </is>
+      </c>
+      <c r="U198" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/20662679</t>
+        </is>
+      </c>
+      <c r="V198" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>헬스장</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>뷰티니스짐 효자지점</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>beautinessgymhyoja@naver.com</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr"/>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>0507-1327-9682</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr"/>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>전북특별자치도 전주시 완산구 효동2길 1 4층</t>
+        </is>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/beautinessgymhyoja</t>
+        </is>
+      </c>
+      <c r="I199" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J199" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K199" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="L199" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M199" t="inlineStr"/>
+      <c r="N199" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O199" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P199" t="n">
+        <v>1960</v>
+      </c>
+      <c r="Q199" t="n">
+        <v>79</v>
+      </c>
+      <c r="R199" t="n">
+        <v>2039</v>
+      </c>
+      <c r="S199" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T199" t="inlineStr">
+        <is>
+          <t>1129813754</t>
+        </is>
+      </c>
+      <c r="U199" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1129813754</t>
+        </is>
+      </c>
+      <c r="V199" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>헬스장</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>베가짐</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>bjk7300@naver.com</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr"/>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>0507-1460-7930</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr"/>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>전북특별자치도 전주시 완산구 서신로 5 지하1층</t>
+        </is>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/vegagym_official_</t>
+        </is>
+      </c>
+      <c r="I200" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J200" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K200" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L200" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M200" t="inlineStr"/>
+      <c r="N200" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O200" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P200" t="n">
+        <v>26</v>
+      </c>
+      <c r="Q200" t="n">
+        <v>5</v>
+      </c>
+      <c r="R200" t="n">
+        <v>31</v>
+      </c>
+      <c r="S200" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T200" t="inlineStr">
+        <is>
+          <t>2087401469</t>
+        </is>
+      </c>
+      <c r="U200" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/2087401469</t>
+        </is>
+      </c>
+      <c r="V200" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>헬스장</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>국가대표휘트니스</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>pkmpowere@naver.com</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr"/>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>0507-1388-1154</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr"/>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>전북특별자치도 전주시 덕진구 안덕원로 276 2동 3층</t>
+        </is>
+      </c>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/kyeongmo.park</t>
+        </is>
+      </c>
+      <c r="I201" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J201" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K201" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L201" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M201" t="inlineStr"/>
+      <c r="N201" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O201" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P201" t="n">
+        <v>1196</v>
+      </c>
+      <c r="Q201" t="n">
+        <v>56</v>
+      </c>
+      <c r="R201" t="n">
+        <v>1252</v>
+      </c>
+      <c r="S201" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T201" t="inlineStr">
+        <is>
+          <t>1276713609</t>
+        </is>
+      </c>
+      <c r="U201" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1276713609</t>
+        </is>
+      </c>
+      <c r="V201" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>스포츠시설</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>바디플랜짐</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>plangym1@naver.com</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr"/>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>0507-1369-8691</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr"/>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>전북특별자치도 전주시 완산구 여울로 35 7층 바디플랜짐</t>
+        </is>
+      </c>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/bodyplan_gym</t>
+        </is>
+      </c>
+      <c r="I202" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J202" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K202" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L202" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M202" t="inlineStr"/>
+      <c r="N202" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O202" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P202" t="n">
+        <v>14</v>
+      </c>
+      <c r="Q202" t="n">
+        <v>160</v>
+      </c>
+      <c r="R202" t="n">
+        <v>174</v>
+      </c>
+      <c r="S202" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T202" t="inlineStr">
+        <is>
+          <t>1945263108</t>
+        </is>
+      </c>
+      <c r="U202" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1945263108</t>
+        </is>
+      </c>
+      <c r="V202" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>